<commit_message>
Add Invoices intake tab + invoice-automation setup guide
New Invoices tab is the target for the Outlook->Excel Power Automate flow
(kept separate from Owl Ops Tasks). Trends now splits task counts (from
Tasks) and cost charts (from Invoices), so cost populates as invoices flow
in. Adds Invoice_Robot_Setup.md, a plain-language one-time setup walkthrough.

https://claude.ai/code/session_016MSrojN6N6Hir9VZegfpJa
</commit_message>
<xml_diff>
--- a/Invoice_Tracker_Template.xlsx
+++ b/Invoice_Tracker_Template.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="START HERE" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Tasks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Stores" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Equipment Types" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Trends" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Invoices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Stores" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Equipment Types" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Trends" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="StoreList">Stores!$A$2:$A$500</definedName>
@@ -59,7 +60,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +70,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -109,6 +115,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -277,7 +286,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Open Tasks by Equipment Type</a:t>
+              <a:t>Invoice Cost by Store ($)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -285,14 +294,14 @@
     </title>
     <plotArea>
       <barChart>
-        <barDir val="bar"/>
+        <barDir val="col"/>
         <grouping val="clustered"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Trends'!F5</f>
+              <f>'Trends'!C5</f>
             </strRef>
           </tx>
           <spPr>
@@ -302,12 +311,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Trends'!$E$6:$E$12</f>
+              <f>'Trends'!$A$6:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Trends'!$F$6:$F$12</f>
+              <f>'Trends'!$C$6:$C$10</f>
             </numRef>
           </val>
         </ser>
@@ -356,7 +365,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Cost by Month ($) — fills in as invoices arrive</a:t>
+              <a:t>Invoice Cost by Month ($)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -429,11 +438,90 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Open Tasks by Equipment</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Trends'!F5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Trends'!$E$6:$E$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Trends'!$F$6:$F$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -455,12 +543,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>8</col>
       <colOff>0</colOff>
       <row>19</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4320000" cy="3240000"/>
+    <ext cx="4320000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -477,7 +565,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>15</col>
+      <col>16</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -492,6 +580,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>16</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4320000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -527,7 +637,28 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblStores" displayName="tblStores" ref="A1:C6" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblInvoices" displayName="tblInvoices" ref="A1:L2" headerRowCount="1">
+  <autoFilter ref="A1:L2"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="Invoice Date"/>
+    <tableColumn id="2" name="Month"/>
+    <tableColumn id="3" name="Store"/>
+    <tableColumn id="4" name="Equipment Type"/>
+    <tableColumn id="5" name="Cost ($)"/>
+    <tableColumn id="6" name="Vendor"/>
+    <tableColumn id="7" name="Invoice #"/>
+    <tableColumn id="8" name="Description"/>
+    <tableColumn id="9" name="Status"/>
+    <tableColumn id="10" name="Source (email)"/>
+    <tableColumn id="11" name="Date Captured"/>
+    <tableColumn id="12" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblStores" displayName="tblStores" ref="A1:C6" headerRowCount="1">
   <autoFilter ref="A1:C6"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Store"/>
@@ -538,9 +669,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblEquip" displayName="tblEquip" ref="A1:B24" headerRowCount="1">
-  <autoFilter ref="A1:B24"/>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblEquip" displayName="tblEquip" ref="A1:B25" headerRowCount="1">
+  <autoFilter ref="A1:B25"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Equipment Type"/>
     <tableColumn id="2" name="Class"/>
@@ -838,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B18"/>
+  <dimension ref="B1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -855,7 +986,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Built from your Owl Ops export. Columns now match your real data.</t>
+          <t>Two sources, one tracker. Your Owl Ops tasks + your Outlook invoices.</t>
         </is>
       </c>
     </row>
@@ -872,28 +1003,28 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>• Tasks      → your work orders / invoices. Your 9 tasks are already loaded.</t>
+          <t>• Tasks     → from Owl Ops (what broke, where). Your 9 tasks are loaded.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>• Stores     → your locations (auto-filled from the export).</t>
+          <t>• Invoices  → from Outlook. THE ROBOT FILLS THIS automatically once set up.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>• Equipment Types → the drop-down list for the Equipment column.</t>
+          <t>• Stores / Equipment Types → drop-down lists.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>• Trends     → charts: tasks by store, by equipment, and cost (fills in as invoices arrive).</t>
+          <t>• Trends    → charts. Task counts now; cost charts fill as invoices arrive.</t>
         </is>
       </c>
     </row>
@@ -903,55 +1034,21 @@
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>HOW TO ADD MORE</t>
+          <t>THE INVOICE ROBOT</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>• Each new Owl Ops export: send it to me and I'll drop it straight into the Tasks tab,</t>
+          <t>Set it up once (see the setup guide I sent). After that: an invoice hits Outlook →</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  or add rows yourself — Store, Equipment, Priority, Type, Status are drop-downs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>ABOUT COST</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>These are OPEN tasks, so Cost is $0 until a vendor invoices the work. When you get an</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>invoice, type the amount in the Cost column and the Trends cost charts update automatically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>The Equipment Type column is my best guess from each description — please review &amp; fix.</t>
+          <t>a row appears on the Invoices tab by itself. You just glance weekly to set Equipment Type.</t>
         </is>
       </c>
     </row>
@@ -1720,117 +1817,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Invoice Date</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Store</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Region</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Address</t>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Equipment Type</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Cost ($)</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Invoice #</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>Source (email)</t>
+        </is>
+      </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>Date Captured</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>DD National City</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2139 E. Plaza Blvd, National City, California</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DD JJ Convoy</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>4140 Convoy St, San Diego, CA</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DD JJ Montezuma</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>5825 Montezuma Rd,  San Diego, CA</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>DD Washington St</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>409 Washington St, San Diego, CA</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>DD Miramar Flightline</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>8635 Obregon Ave., Bldg 8675, MCAS Miramar, San Diego, California</t>
-        </is>
-      </c>
+      <c r="A2" s="6" t="n"/>
+      <c r="B2">
+        <f>IF($A2="","",TEXT($A2,"YYYY-MM"))</f>
+        <v/>
+      </c>
+      <c r="E2" s="7" t="n"/>
+      <c r="K2" s="6" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=StoreList</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=EquipList</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pending,Approved,Paid,Disputed"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1844,298 +1930,113 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Equipment Type</t>
+          <t>Store</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Class</t>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Address</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fryer</t>
+          <t>DD National City</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cooking</t>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2139 E. Plaza Blvd, National City, California</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Range / Oven</t>
+          <t>DD JJ Convoy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cooking</t>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>4140 Convoy St, San Diego, CA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Grill / Griddle</t>
+          <t>DD JJ Montezuma</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cooking</t>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>5825 Montezuma Rd,  San Diego, CA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hood / Exhaust Fan</t>
+          <t>DD Washington St</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>409 Washington St, San Diego, CA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Walk-in Cooler</t>
+          <t>DD Miramar Flightline</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Refrigeration</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Reach-in Freezer</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Refrigeration</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Ice Machine</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Refrigeration</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Soda / Beverage Fountain</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Beverage</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Coffee Machine</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Beverage</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Blender / Prep Equipment</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Toaster</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Cooking</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Dishwasher</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Warewashing</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Grease Trap</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Plumbing</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Water Heater</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Plumbing</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Rooftop HVAC Unit</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>HVAC</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Mini-split AC</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>HVAC</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>POS Terminal</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>POS / IT</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Receipt Printer</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>POS / IT</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Security / CCTV</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>POS / IT</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Lighting / Electrical</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Electrical</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Plumbing / Restroom</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Plumbing</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Doors / Locks</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Building</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Other</t>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>8635 Obregon Ave., Bldg 8675, MCAS Miramar, San Diego, California</t>
         </is>
       </c>
     </row>
@@ -2153,15 +2054,337 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Equipment Type</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fryer</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cooking</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Range / Oven</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cooking</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Grill / Griddle</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cooking</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hood / Exhaust Fan</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Walk-in Cooler</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Refrigeration</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Reach-in Freezer</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Refrigeration</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ice Machine</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Refrigeration</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Soda / Beverage Fountain</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Beverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Coffee Machine</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Beverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Blender / Prep Equipment</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Toaster</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Cooking</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Dishwasher</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Warewashing</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Grease Trap</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Water Heater</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rooftop HVAC Unit</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mini-split AC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>POS Terminal</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>POS / IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Receipt Printer</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>POS / IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Security / CCTV</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>POS / IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Lighting / Electrical</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Plumbing / Restroom</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Doors / Locks</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Building</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>— set me</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2174,7 +2397,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Live from the Tasks tab.</t>
+          <t>Task counts come from Owl Ops; $ comes from invoices (fills in as the robot runs).</t>
         </is>
       </c>
     </row>
@@ -2191,29 +2414,34 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Store</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t># Open Tasks</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Invoice Cost ($)</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t># Tasks</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Cost ($)</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Equipment</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t># Tasks</t>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Invoice Cost ($)</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2456,7 @@
         <v/>
       </c>
       <c r="C6" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$C$2:$C$5000,$A6)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$C$2:$C$5000,$A6)</f>
         <v/>
       </c>
       <c r="E6" t="inlineStr">
@@ -2240,6 +2468,10 @@
         <f>COUNTIF(Tasks!$O$2:$O$5000,$E6)</f>
         <v/>
       </c>
+      <c r="G6" s="7">
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$D$2:$D$5000,$E6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2252,7 +2484,7 @@
         <v/>
       </c>
       <c r="C7" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$C$2:$C$5000,$A7)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$C$2:$C$5000,$A7)</f>
         <v/>
       </c>
       <c r="E7" t="inlineStr">
@@ -2264,6 +2496,10 @@
         <f>COUNTIF(Tasks!$O$2:$O$5000,$E7)</f>
         <v/>
       </c>
+      <c r="G7" s="7">
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$D$2:$D$5000,$E7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2276,7 +2512,7 @@
         <v/>
       </c>
       <c r="C8" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$C$2:$C$5000,$A8)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$C$2:$C$5000,$A8)</f>
         <v/>
       </c>
       <c r="E8" t="inlineStr">
@@ -2288,6 +2524,10 @@
         <f>COUNTIF(Tasks!$O$2:$O$5000,$E8)</f>
         <v/>
       </c>
+      <c r="G8" s="7">
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$D$2:$D$5000,$E8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2300,7 +2540,7 @@
         <v/>
       </c>
       <c r="C9" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$C$2:$C$5000,$A9)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$C$2:$C$5000,$A9)</f>
         <v/>
       </c>
       <c r="E9" t="inlineStr">
@@ -2312,6 +2552,10 @@
         <f>COUNTIF(Tasks!$O$2:$O$5000,$E9)</f>
         <v/>
       </c>
+      <c r="G9" s="7">
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$D$2:$D$5000,$E9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2324,7 +2568,7 @@
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$C$2:$C$5000,$A10)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$C$2:$C$5000,$A10)</f>
         <v/>
       </c>
       <c r="E10" t="inlineStr">
@@ -2336,6 +2580,10 @@
         <f>COUNTIF(Tasks!$O$2:$O$5000,$E10)</f>
         <v/>
       </c>
+      <c r="G10" s="7">
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$D$2:$D$5000,$E10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="E11" t="inlineStr">
@@ -2347,11 +2595,15 @@
         <f>COUNTIF(Tasks!$O$2:$O$5000,$E11)</f>
         <v/>
       </c>
+      <c r="G11" s="7">
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$D$2:$D$5000,$E11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Cost by Month</t>
+          <t>Invoice Cost by Month</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2363,14 +2615,18 @@
         <f>COUNTIF(Tasks!$O$2:$O$5000,$E12)</f>
         <v/>
       </c>
+      <c r="G12" s="7">
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$D$2:$D$5000,$E12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Cost ($)</t>
         </is>
@@ -2383,7 +2639,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A14)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A14)</f>
         <v/>
       </c>
     </row>
@@ -2394,7 +2650,7 @@
         </is>
       </c>
       <c r="B15" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A15)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A15)</f>
         <v/>
       </c>
     </row>
@@ -2405,7 +2661,7 @@
         </is>
       </c>
       <c r="B16" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A16)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A16)</f>
         <v/>
       </c>
     </row>
@@ -2416,7 +2672,7 @@
         </is>
       </c>
       <c r="B17" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A17)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A17)</f>
         <v/>
       </c>
     </row>
@@ -2427,7 +2683,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A18)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A18)</f>
         <v/>
       </c>
     </row>
@@ -2438,7 +2694,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A19)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A19)</f>
         <v/>
       </c>
     </row>
@@ -2449,7 +2705,7 @@
         </is>
       </c>
       <c r="B20" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A20)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A20)</f>
         <v/>
       </c>
     </row>
@@ -2460,7 +2716,7 @@
         </is>
       </c>
       <c r="B21" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A21)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A21)</f>
         <v/>
       </c>
     </row>
@@ -2471,7 +2727,7 @@
         </is>
       </c>
       <c r="B22" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A22)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A22)</f>
         <v/>
       </c>
     </row>
@@ -2482,7 +2738,7 @@
         </is>
       </c>
       <c r="B23" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A23)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A23)</f>
         <v/>
       </c>
     </row>
@@ -2493,7 +2749,7 @@
         </is>
       </c>
       <c r="B24" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A24)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A24)</f>
         <v/>
       </c>
     </row>
@@ -2504,7 +2760,7 @@
         </is>
       </c>
       <c r="B25" s="7">
-        <f>SUMIFS(Tasks!$I$2:$I$5000,Tasks!$P$2:$P$5000,$A25)</f>
+        <f>SUMIFS(Invoices!$E$2:$E$5000,Invoices!$B$2:$B$5000,$A25)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Embed setup guide as START HERE sheet; remove .md dependency
https://claude.ai/code/session_016MSrojN6N6Hir9VZegfpJa
</commit_message>
<xml_diff>
--- a/Invoice_Tracker_Template.xlsx
+++ b/Invoice_Tracker_Template.xlsx
@@ -27,7 +27,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +58,28 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00888888"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00222222"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -104,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +141,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -969,90 +1015,314 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B12"/>
+  <dimension ref="B1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="82" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Equipment &amp; Repair Tracker</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Two sources, one tracker. Your Owl Ops tasks + your Outlook invoices.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>THE TABS</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>• Tasks     → from Owl Ops (what broke, where). Your 9 tasks are loaded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>• Invoices  → from Outlook. THE ROBOT FILLS THIS automatically once set up.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>• Stores / Equipment Types → drop-down lists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>• Trends    → charts. Task counts now; cost charts fill as invoices arrive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>THE INVOICE ROBOT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Set it up once (see the setup guide I sent). After that: an invoice hits Outlook →</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>a row appears on the Invoices tab by itself. You just glance weekly to set Equipment Type.</t>
+    <row r="1" ht="30" customHeight="1">
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Invoice Robot — One-Time Setup Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="B2" s="11" t="inlineStr"/>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Do this once (~30 min). After that, invoices fill the tracker automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>BEFORE YOU START</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>1.  Save tracker to OneDrive</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Open this file → File → Save As → OneDrive. The robot needs it in the cloud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>2.  Make an Outlook folder</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>In Outlook → right-click your Inbox → New Folder → name it  Invoices</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>3.  Make an Outlook rule</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Outlook → Settings → Rules → New rule → 'If subject contains invoice' → Move to Invoices folder → Save</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="8" customHeight="1"/>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>BUILD THE ROBOT  (go to: make.powerautomate.com — sign in with your work email)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="4" customHeight="1"/>
+    <row r="11" ht="52" customHeight="1">
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Step 1</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Left menu → click  + Create  →  Automated cloud flow
+Flow name: Invoice to Tracker
+Search for:  When a new email arrives (V3)  → click it → Create</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Step 2</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>In the trigger box:
+• Folder → folder icon → choose  Invoices
+• Click  Show advanced options  →  Only with Attachments: Yes   and   Include Attachments: Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="52" customHeight="1">
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Step 3</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Click + → Add an action → search:  Extract information from invoices  → click it
+(If it offers an AI Builder trial → click Yes, it's free for 30 days)
+In the  Invoice file  box → click the ⚡ lightning bolt → choose  Attachments Content
+A grey 'Apply to each' box appears — that's normal, leave it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Step 4</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>INSIDE the grey box → click + → Add an action
+Search:  Add a row into a table  → pick the  Excel Online (Business)  one
+• Location: OneDrive for Business   • Library: OneDrive
+• File: browse to this tracker   • Table: tblInvoices</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Fill the column boxes — click ⚡ in each box to pick the value:
+• Invoice Date  → Invoice date
+• Cost ($)  → Invoice total (the number one, not the text one)
+• Vendor  → Vendor name
+• Invoice #  → Invoice ID
+• Store  → Service address
+• Equipment Type  → just type the word:  Review
+• Status  → just type:  Pending
+• Date Captured  → ⚡ → Expression tab → type  utcNow()  → OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Step 6</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>Click  Save  (top right corner).  Done — the robot is live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="8" customHeight="1"/>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>TEST IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="14" t="inlineStr"/>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Forward yourself any invoice PDF so it lands in the Outlook Invoices folder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="14" t="inlineStr"/>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>Wait ~1 minute → open this file → click the Invoices tab → a new row should be there. ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="8" customHeight="1"/>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>WHAT'S AUTOMATIC vs. YOUR 10 SECONDS/WEEK</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Robot does automatically →</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Date · Cost · Vendor · Invoice # · drops the row · charts update themselves</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>You do (~10 sec per invoice) →</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>Open Invoices tab → pick Equipment Type from the dropdown in column D → confirm Store in column C</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="8" customHeight="1"/>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>TROUBLESHOOTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>No row appeared?</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>Power Automate → My flows → click your flow → Run history → tell me what the red X says</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>Invoices in email body not PDF?</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>Tell me — Step 3 changes slightly. Takes 2 min to adjust.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>AI Builder cost after trial?</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>~$40/mo for the plan. If that's a problem tell me — I have a no-cost workaround.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="8" customHeight="1"/>
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>OWL OPS TASKS (the other source)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>For now →</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>Each week: export from Owl Ops → send me the CSV → I load the new tasks in for you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>To automate it →</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>Look in Owl Ops Reports for a 'Schedule' or 'Email report' button. If it exists, tell me and I'll wire that up too.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B18:C18"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1206,7 +1476,6 @@
           <t>Michael Rivas</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" s="7" t="n">
         <v>0</v>
       </c>
@@ -1238,7 +1507,6 @@
         <f>IF($F2="","",TEXT($F2,"YYYY-MM"))</f>
         <v/>
       </c>
-      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1274,7 +1542,6 @@
           <t>Ivan Gonzalez</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" s="7" t="n">
         <v>0</v>
       </c>
@@ -1306,7 +1573,6 @@
         <f>IF($F3="","",TEXT($F3,"YYYY-MM"))</f>
         <v/>
       </c>
-      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1342,7 +1608,6 @@
           <t>Junior Berumen</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" s="7" t="n">
         <v>0</v>
       </c>
@@ -1374,7 +1639,6 @@
         <f>IF($F4="","",TEXT($F4,"YYYY-MM"))</f>
         <v/>
       </c>
-      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1410,7 +1674,6 @@
           <t>Junior Berumen</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" s="7" t="n">
         <v>0</v>
       </c>
@@ -1442,7 +1705,6 @@
         <f>IF($F5="","",TEXT($F5,"YYYY-MM"))</f>
         <v/>
       </c>
-      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1478,7 +1740,6 @@
           <t>Junior Berumen</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" s="7" t="n">
         <v>0</v>
       </c>
@@ -1510,7 +1771,6 @@
         <f>IF($F6="","",TEXT($F6,"YYYY-MM"))</f>
         <v/>
       </c>
-      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1546,7 +1806,6 @@
           <t>Catherine Corcoran</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" s="7" t="n">
         <v>0</v>
       </c>
@@ -1580,7 +1839,6 @@
         <f>IF($F7="","",TEXT($F7,"YYYY-MM"))</f>
         <v/>
       </c>
-      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1616,7 +1874,6 @@
           <t>Michael Rivas</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" s="7" t="n">
         <v>0</v>
       </c>
@@ -1648,7 +1905,6 @@
         <f>IF($F8="","",TEXT($F8,"YYYY-MM"))</f>
         <v/>
       </c>
-      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1684,7 +1940,6 @@
           <t>Jackie Gomez</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" s="7" t="n">
         <v>0</v>
       </c>
@@ -1716,7 +1971,6 @@
         <f>IF($F9="","",TEXT($F9,"YYYY-MM"))</f>
         <v/>
       </c>
-      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1752,7 +2006,6 @@
           <t>Ivan Gonzalez</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" s="7" t="n">
         <v>0</v>
       </c>
@@ -1784,7 +2037,6 @@
         <f>IF($F10="","",TEXT($F10,"YYYY-MM"))</f>
         <v/>
       </c>
-      <c r="Q10" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="5">

</xml_diff>